<commit_message>
CPO-672 정산명세 추가 2026-06-16 16:30
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260616.xlsx
+++ b/RNR_수입원가_2026_20260616.xlsx
@@ -17157,14 +17157,14 @@
         <v>46189</v>
       </c>
       <c r="N16" s="278" t="n">
-        <v>1517.2</v>
+        <v>1517.25</v>
       </c>
       <c r="O16" s="281" t="n">
         <v>336629315</v>
       </c>
       <c r="P16" s="276" t="inlineStr">
         <is>
-          <t>6/16 만기 상환 완료 (외국환 거래표 2026-06-16, REF M88JX2510NU00018). 원금 USD 221,868.99 → 원화 336,629,315 (적용환율 1,517.20). 미결제잔액 USD 0.00</t>
+          <t>6/16 만기 상환 완료 (외국환 거래표 2026-06-16, REF M88JX2510NU00018). 원금 USD 221,868.00 → 원화 336,629,315 (적용환율 1,517.25, 은행 실제 출금액). 미결제잔액 USD 0.00, 하단 정산 명세 참조</t>
         </is>
       </c>
     </row>
@@ -18128,25 +18128,536 @@
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
-    <row r="49" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="50" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="51" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="52" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="53" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="54" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="55" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="56" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="57" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="58" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="59" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="60" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="61" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="62" ht="15.75" customFormat="1" customHeight="1" s="160"/>
-    <row r="63" ht="15.75" customFormat="1" customHeight="1" s="160"/>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="A45" s="252" t="inlineStr">
+        <is>
+          <t>&lt; CPO-672 상환 정산 및 수수료 명세 (신한은행, 출처: 은행 수수료/인도 내역서 2026-06-16) &gt;</t>
+        </is>
+      </c>
+      <c r="B45" s="65" t="n"/>
+      <c r="C45" s="66" t="n"/>
+      <c r="D45" s="65" t="n"/>
+      <c r="E45" s="65" t="n"/>
+      <c r="F45" s="65" t="n"/>
+      <c r="G45" s="65" t="n"/>
+      <c r="H45" s="65" t="n"/>
+      <c r="I45" s="65" t="n"/>
+      <c r="J45" s="65" t="n"/>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="A46" s="253" t="inlineStr">
+        <is>
+          <t>상환일</t>
+        </is>
+      </c>
+      <c r="B46" s="253" t="inlineStr">
+        <is>
+          <t>상환원금(USD)</t>
+        </is>
+      </c>
+      <c r="C46" s="253" t="inlineStr">
+        <is>
+          <t>상환환율(₩)</t>
+        </is>
+      </c>
+      <c r="D46" s="253" t="inlineStr">
+        <is>
+          <t>상환금액(KRW)</t>
+        </is>
+      </c>
+      <c r="E46" s="253" t="inlineStr">
+        <is>
+          <t>L/C No.</t>
+        </is>
+      </c>
+      <c r="F46" s="253" t="inlineStr">
+        <is>
+          <t>회계처리(권장)</t>
+        </is>
+      </c>
+      <c r="G46" s="65" t="n"/>
+      <c r="H46" s="65" t="n"/>
+      <c r="I46" s="65" t="n"/>
+      <c r="J46" s="65" t="n"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="A47" s="254" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B47" s="255" t="n">
+        <v>221868</v>
+      </c>
+      <c r="C47" s="255" t="n">
+        <v>1517.25</v>
+      </c>
+      <c r="D47" s="264" t="n">
+        <v>336629315</v>
+      </c>
+      <c r="E47" s="257" t="inlineStr">
+        <is>
+          <t>M88JX2510NU00018</t>
+        </is>
+      </c>
+      <c r="F47" s="258" t="inlineStr">
+        <is>
+          <t>차변 외화매입채무(USANCE) 221,868 USD 제거 + 외환차손익, 대변 보통예금 336,629,315</t>
+        </is>
+      </c>
+      <c r="G47" s="71" t="n"/>
+      <c r="H47" s="65" t="n"/>
+      <c r="I47" s="65" t="n"/>
+      <c r="J47" s="65" t="n"/>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" s="65" t="n"/>
+      <c r="B48" s="65" t="n"/>
+      <c r="C48" s="66" t="n"/>
+      <c r="D48" s="65" t="n"/>
+      <c r="E48" s="65" t="n"/>
+      <c r="F48" s="70" t="n"/>
+      <c r="G48" s="71" t="n"/>
+      <c r="H48" s="65" t="n"/>
+      <c r="I48" s="65" t="n"/>
+      <c r="J48" s="65" t="n"/>
+    </row>
+    <row r="49" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A49" s="253" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B49" s="253" t="inlineStr">
+        <is>
+          <t>징수일</t>
+        </is>
+      </c>
+      <c r="C49" s="253" t="inlineStr">
+        <is>
+          <t>수수료 구분</t>
+        </is>
+      </c>
+      <c r="D49" s="253" t="inlineStr">
+        <is>
+          <t>이율(%)</t>
+        </is>
+      </c>
+      <c r="E49" s="253" t="inlineStr">
+        <is>
+          <t>수수료 기간</t>
+        </is>
+      </c>
+      <c r="F49" s="259" t="inlineStr">
+        <is>
+          <t>일수</t>
+        </is>
+      </c>
+      <c r="G49" s="260" t="inlineStr">
+        <is>
+          <t>대상금액(USD)</t>
+        </is>
+      </c>
+      <c r="H49" s="253" t="inlineStr">
+        <is>
+          <t>USD 상당액</t>
+        </is>
+      </c>
+      <c r="I49" s="253" t="inlineStr">
+        <is>
+          <t>징수액(KRW)</t>
+        </is>
+      </c>
+      <c r="J49" s="253" t="inlineStr">
+        <is>
+          <t>회계처리(권장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A50" s="257" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" s="254" t="n">
+        <v>45946</v>
+      </c>
+      <c r="C50" s="261" t="inlineStr">
+        <is>
+          <t>수입신용장 기간수수료(발행수수료, 360일 단위)</t>
+        </is>
+      </c>
+      <c r="D50" s="262" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E50" s="257" t="inlineStr">
+        <is>
+          <t>2025-10-16 ~ 2025-12-19</t>
+        </is>
+      </c>
+      <c r="F50" s="263" t="n">
+        <v>65</v>
+      </c>
+      <c r="G50" s="255" t="n">
+        <v>221868</v>
+      </c>
+      <c r="H50" s="255" t="n">
+        <v>320.46</v>
+      </c>
+      <c r="I50" s="264" t="n">
+        <v>454691</v>
+      </c>
+      <c r="J50" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A51" s="257" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="254" t="n">
+        <v>45946</v>
+      </c>
+      <c r="C51" s="261" t="inlineStr">
+        <is>
+          <t>전신료(일반신용장 USANCE)</t>
+        </is>
+      </c>
+      <c r="D51" s="262" t="n"/>
+      <c r="E51" s="257" t="inlineStr"/>
+      <c r="F51" s="263" t="n">
+        <v>0</v>
+      </c>
+      <c r="G51" s="255" t="n"/>
+      <c r="H51" s="255" t="n"/>
+      <c r="I51" s="264" t="n">
+        <v>13750</v>
+      </c>
+      <c r="J51" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A52" s="257" t="n">
+        <v>3</v>
+      </c>
+      <c r="B52" s="254" t="n">
+        <v>45961</v>
+      </c>
+      <c r="C52" s="261" t="inlineStr">
+        <is>
+          <t>수입화물선취보증서(L/G) 발급수수료</t>
+        </is>
+      </c>
+      <c r="D52" s="262" t="n"/>
+      <c r="E52" s="257" t="inlineStr"/>
+      <c r="F52" s="263" t="n">
+        <v>0</v>
+      </c>
+      <c r="G52" s="255" t="n"/>
+      <c r="H52" s="255" t="n"/>
+      <c r="I52" s="264" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J52" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A53" s="257" t="n">
+        <v>4</v>
+      </c>
+      <c r="B53" s="254" t="n">
+        <v>46007</v>
+      </c>
+      <c r="C53" s="261" t="inlineStr">
+        <is>
+          <t>수입화물선취보증료(외화)</t>
+        </is>
+      </c>
+      <c r="D53" s="262" t="n">
+        <v>3</v>
+      </c>
+      <c r="E53" s="257" t="inlineStr">
+        <is>
+          <t>2025-10-31 ~ 2025-12-15</t>
+        </is>
+      </c>
+      <c r="F53" s="263" t="n">
+        <v>46</v>
+      </c>
+      <c r="G53" s="255" t="n">
+        <v>221868</v>
+      </c>
+      <c r="H53" s="255" t="n">
+        <v>850.55</v>
+      </c>
+      <c r="I53" s="264" t="n">
+        <v>1255244</v>
+      </c>
+      <c r="J53" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A54" s="257" t="n">
+        <v>5</v>
+      </c>
+      <c r="B54" s="254" t="n">
+        <v>46007</v>
+      </c>
+      <c r="C54" s="261" t="inlineStr">
+        <is>
+          <t>수입인수수수료(360일 단위)</t>
+        </is>
+      </c>
+      <c r="D54" s="262" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E54" s="257" t="inlineStr">
+        <is>
+          <t>2025-12-16 ~ 2026-06-14</t>
+        </is>
+      </c>
+      <c r="F54" s="263" t="n">
+        <v>181</v>
+      </c>
+      <c r="G54" s="255" t="n">
+        <v>221868</v>
+      </c>
+      <c r="H54" s="255" t="n">
+        <v>1338.62</v>
+      </c>
+      <c r="I54" s="264" t="n">
+        <v>1975645</v>
+      </c>
+      <c r="J54" s="257" t="inlineStr">
+        <is>
+          <t>이자비용</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A55" s="257" t="n">
+        <v>6</v>
+      </c>
+      <c r="B55" s="254" t="n">
+        <v>46007</v>
+      </c>
+      <c r="C55" s="261" t="inlineStr">
+        <is>
+          <t>수입기간수수료 환급(-)</t>
+        </is>
+      </c>
+      <c r="D55" s="262" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="E55" s="257" t="inlineStr">
+        <is>
+          <t>2025-12-16 ~ 2025-12-19</t>
+        </is>
+      </c>
+      <c r="F55" s="263" t="n">
+        <v>4</v>
+      </c>
+      <c r="G55" s="255" t="n">
+        <v>221868</v>
+      </c>
+      <c r="H55" s="255" t="n">
+        <v>-19.72</v>
+      </c>
+      <c r="I55" s="264" t="n">
+        <v>-27981</v>
+      </c>
+      <c r="J55" s="257" t="inlineStr">
+        <is>
+          <t>지급수수료 차감</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A56" s="257" t="n">
+        <v>7</v>
+      </c>
+      <c r="B56" s="254" t="n">
+        <v>46189</v>
+      </c>
+      <c r="C56" s="261" t="inlineStr">
+        <is>
+          <t>수입인수수수료(만기연장 1일분)</t>
+        </is>
+      </c>
+      <c r="D56" s="262" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E56" s="257" t="inlineStr">
+        <is>
+          <t>2026-06-15 ~ 2026-06-15</t>
+        </is>
+      </c>
+      <c r="F56" s="263" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="255" t="n">
+        <v>221868</v>
+      </c>
+      <c r="H56" s="255" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="I56" s="264" t="n">
+        <v>11186</v>
+      </c>
+      <c r="J56" s="257" t="inlineStr">
+        <is>
+          <t>이자비용</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A57" s="257" t="n">
+        <v>8</v>
+      </c>
+      <c r="B57" s="254" t="n">
+        <v>46189</v>
+      </c>
+      <c r="C57" s="261" t="inlineStr">
+        <is>
+          <t>해외수수료(해외은행 인수금융 이자)</t>
+        </is>
+      </c>
+      <c r="D57" s="262" t="n"/>
+      <c r="E57" s="257" t="inlineStr">
+        <is>
+          <t>2025-12-19 인도 ~ 2026-06-16</t>
+        </is>
+      </c>
+      <c r="F57" s="263" t="n">
+        <v>180</v>
+      </c>
+      <c r="G57" s="255" t="n">
+        <v>221868</v>
+      </c>
+      <c r="H57" s="255" t="n">
+        <v>6124.77</v>
+      </c>
+      <c r="I57" s="264" t="n">
+        <v>9292540</v>
+      </c>
+      <c r="J57" s="257" t="inlineStr">
+        <is>
+          <t>이자비용</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A58" s="253" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+      <c r="B58" s="265" t="n"/>
+      <c r="C58" s="266" t="n"/>
+      <c r="D58" s="265" t="n"/>
+      <c r="E58" s="265" t="n"/>
+      <c r="F58" s="265" t="n"/>
+      <c r="G58" s="268" t="n"/>
+      <c r="H58" s="269" t="n">
+        <v>8622.08</v>
+      </c>
+      <c r="I58" s="270" t="n">
+        <v>12980075</v>
+      </c>
+      <c r="J58" s="253" t="inlineStr">
+        <is>
+          <t>이자비용 11,279,371 + 지급수수료 1,700,704</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A59" s="274" t="inlineStr">
+        <is>
+          <t>주1: USD 상당액 = 대상금액 x 이율 x 일수/360 (전신료, L/G 발급료는 KRW 정액)</t>
+        </is>
+      </c>
+      <c r="B59" s="65" t="n"/>
+      <c r="C59" s="66" t="n"/>
+      <c r="D59" s="65" t="n"/>
+      <c r="E59" s="65" t="n"/>
+      <c r="F59" s="65" t="n"/>
+      <c r="G59" s="71" t="n"/>
+      <c r="H59" s="65" t="n"/>
+      <c r="I59" s="65" t="n"/>
+      <c r="J59" s="65" t="n"/>
+    </row>
+    <row r="60" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A60" s="274" t="inlineStr">
+        <is>
+          <t>주2: No.1~6 수수료는 징수일에 KRW 기징수, No.7(만기연장)·해외수수료는 상환일(6/16) 출금. 회계처리는 각 징수일자 전표로 계상</t>
+        </is>
+      </c>
+      <c r="B60" s="65" t="n"/>
+      <c r="C60" s="66" t="n"/>
+      <c r="D60" s="65" t="n"/>
+      <c r="E60" s="65" t="n"/>
+      <c r="F60" s="65" t="n"/>
+      <c r="G60" s="71" t="n"/>
+      <c r="H60" s="65" t="n"/>
+      <c r="I60" s="65" t="n"/>
+      <c r="J60" s="65" t="n"/>
+    </row>
+    <row r="61" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A61" s="274" t="inlineStr">
+        <is>
+          <t>주3: 원금 상환 (외국환 거래표 2026-06-16, REF M88JX2510NU00018): 원금 USD 221,868.00 x 적용환율 1,517.25 = 원화 336,629,315 (은행 실제 출금액)</t>
+        </is>
+      </c>
+      <c r="B61" s="65" t="n"/>
+      <c r="C61" s="66" t="n"/>
+      <c r="D61" s="65" t="n"/>
+      <c r="E61" s="65" t="n"/>
+      <c r="F61" s="65" t="n"/>
+      <c r="G61" s="71" t="n"/>
+      <c r="H61" s="65" t="n"/>
+      <c r="I61" s="65" t="n"/>
+      <c r="J61" s="65" t="n"/>
+    </row>
+    <row r="62" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A62" s="274" t="inlineStr">
+        <is>
+          <t>주4: 6/16 실제 출금 합계 345,933,041원 = 원금 336,629,315 + 만기연장 인수수수료 11,186 + 해외수수료 9,292,540</t>
+        </is>
+      </c>
+      <c r="B62" s="65" t="n"/>
+      <c r="C62" s="66" t="n"/>
+      <c r="D62" s="65" t="n"/>
+      <c r="E62" s="65" t="n"/>
+      <c r="F62" s="65" t="n"/>
+      <c r="G62" s="71" t="n"/>
+      <c r="H62" s="65" t="n"/>
+      <c r="I62" s="65" t="n"/>
+      <c r="J62" s="65" t="n"/>
+    </row>
+    <row r="63" ht="15.75" customFormat="1" customHeight="1" s="160">
+      <c r="A63" s="274" t="inlineStr">
+        <is>
+          <t>주5: 해외수수료 KRW 9,292,540은 USD 6,124.77 x 1,517.20 환산 추정 (은행 명세상 KRW 미표기). lcCustomsData 해외수수료(USD 6,124.77)와 일치</t>
+        </is>
+      </c>
+      <c r="B63" s="65" t="n"/>
+      <c r="C63" s="66" t="n"/>
+      <c r="D63" s="65" t="n"/>
+      <c r="E63" s="65" t="n"/>
+      <c r="F63" s="65" t="n"/>
+      <c r="G63" s="71" t="n"/>
+      <c r="H63" s="65" t="n"/>
+      <c r="I63" s="65" t="n"/>
+      <c r="J63" s="65" t="n"/>
+    </row>
     <row r="64" ht="15.75" customFormat="1" customHeight="1" s="160"/>
     <row r="65" ht="15.75" customHeight="1"/>
     <row r="66" ht="15.75" customHeight="1"/>

</xml_diff>